<commit_message>
Flag price and PO differences against Excel; draw Split pages as mini pages
Reconcile
- Read the PO number from each invoice (beside or under its label; never a
  PO Box, a date or an amount) and find PO and amount columns in the sheet.
- Compare every matched invoice with its row: "Price differs" and "PO
  differs" statuses, Amount/Difference/PO columns next to the numbers, a
  count above the table, and a note saying by how much and which way.
  POs compare without prefixes or punctuation; half a cent is rounding.
- Sample register gains a PO column with one wrong amount and one wrong PO.

Split
- Page tiles drawn as tiny pages: a coloured letterhead on an invoice's
  first page, tinted sheets after it, numbers printed on the page; softer
  invoice cards that lift on hover.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/samples/invoice-register.xlsx
+++ b/public/samples/invoice-register.xlsx
@@ -65,9 +65,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,15 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F19"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="9.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,9 +414,12 @@
         <v>Invoice Date</v>
       </c>
       <c r="E1" t="str">
+        <v>PO Number</v>
+      </c>
+      <c r="F1" t="str">
         <v>Amount</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Status</v>
       </c>
     </row>
@@ -442,10 +436,13 @@
       <c r="D2" t="str">
         <v>2026-09-02</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" t="str">
+        <v>4500118</v>
+      </c>
+      <c r="F2">
         <v>1297.48</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -462,10 +459,13 @@
       <c r="D3" t="str">
         <v>2026-09-03</v>
       </c>
-      <c r="E3" s="1">
-        <v>363.96</v>
-      </c>
-      <c r="F3" t="str">
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3">
+        <v>336.96</v>
+      </c>
+      <c r="G3" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -482,10 +482,13 @@
       <c r="D4" t="str">
         <v>2026-09-05</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" t="str">
+        <v>PC-7781</v>
+      </c>
+      <c r="F4">
         <v>716.82</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -502,10 +505,13 @@
       <c r="D5" t="str">
         <v>2026-09-05</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" t="str">
+        <v>PC-7781</v>
+      </c>
+      <c r="F5">
         <v>716.82</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -522,10 +528,13 @@
       <c r="D6" t="str">
         <v>2026-09-08</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" t="str">
+        <v>55103388</v>
+      </c>
+      <c r="F6">
         <v>871.07</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -542,10 +551,13 @@
       <c r="D7" t="str">
         <v>2026-09-10</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7">
         <v>114.91</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -562,10 +574,13 @@
       <c r="D8" t="str">
         <v>2026-09-15</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" t="str">
+        <v>PC-7709</v>
+      </c>
+      <c r="F8">
         <v>1398.73</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -582,10 +597,13 @@
       <c r="D9" t="str">
         <v>2026-09-18</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9">
         <v>146.02</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -602,10 +620,13 @@
       <c r="D10" t="str">
         <v>2026-09-21</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" t="str">
+        <v>PO-4500163</v>
+      </c>
+      <c r="F10">
         <v>187.06</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -622,10 +643,13 @@
       <c r="D11" t="str">
         <v>2026-09-24</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11">
         <v>934.63</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -642,10 +666,13 @@
       <c r="D12" t="str">
         <v>2026-09-26</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12">
         <v>716.82</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -662,10 +689,13 @@
       <c r="D13" t="str">
         <v>2026-09-27</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" t="str">
+        <v>PO 55103401</v>
+      </c>
+      <c r="F13">
         <v>215.35</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -682,10 +712,13 @@
       <c r="D14" t="str">
         <v>2026-09-29</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14">
         <v>298.08</v>
       </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -702,10 +735,13 @@
       <c r="D15" t="str">
         <v>2026-09-30</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15">
         <v>207.36</v>
       </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -722,10 +758,13 @@
       <c r="D16" t="str">
         <v>2026-10-01</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16">
         <v>169.13</v>
       </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -742,10 +781,13 @@
       <c r="D17" t="str">
         <v>2026-10-02</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17">
         <v>822.66</v>
       </c>
-      <c r="F17" t="str">
+      <c r="G17" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -762,10 +804,13 @@
       <c r="D18" t="str">
         <v>2026-10-03</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18">
         <v>248.4</v>
       </c>
-      <c r="F18" t="str">
+      <c r="G18" t="str">
         <v>Open</v>
       </c>
     </row>
@@ -782,16 +827,19 @@
       <c r="D19" t="str">
         <v>2026-10-06</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19">
         <v>412.3</v>
       </c>
-      <c r="F19" t="str">
+      <c r="G19" t="str">
         <v>Open</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>